<commit_message>
Remove files unrelated to the BCP dashboard project
- Drop the separate HR Employee Distribution Heatmap project
  (HR_Heatmap_Dashboard.html, v2, and its geo_hc_by_province export)
- Drop superseded 2026-08-22 geography snapshot and its map image,
  superseded by the 2026-08-23 version
- Remove local .venv/ and desktop.ini clutter (not tracked, but were staged)
</commit_message>
<xml_diff>
--- a/Heatmap.xlsx
+++ b/Heatmap.xlsx
@@ -1155,9 +1155,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B84A1D994D2BDF4995E060F32F257A29" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a13cf0b665a8ae77d7450671e4655040">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="303f9a3f-8d70-4d57-ad77-94345ac92144" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d655ac053d8a2579746362237515854" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B84A1D994D2BDF4995E060F32F257A29" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc917a9190c418ef1116248927f0e9d2">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="303f9a3f-8d70-4d57-ad77-94345ac92144" xmlns:ns3="c77e8c6b-f803-4d24-b07d-f9b9380d87c8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ab56b205e53f2a8c8b8263d1c3412e6" ns2:_="" ns3:_="">
     <xsd:import namespace="303f9a3f-8d70-4d57-ad77-94345ac92144"/>
+    <xsd:import namespace="c77e8c6b-f803-4d24-b07d-f9b9380d87c8"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1167,6 +1168,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1191,6 +1197,43 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="30028c23-345d-4754-af14-b6b609efcc82" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c77e8c6b-f803-4d24-b07d-f9b9380d87c8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{4b9339ab-5444-4089-9db4-1239b440e7b3}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="c77e8c6b-f803-4d24-b07d-f9b9380d87c8">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -1303,12 +1346,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="c77e8c6b-f803-4d24-b07d-f9b9380d87c8" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="303f9a3f-8d70-4d57-ad77-94345ac92144">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5448C89-74A1-48B9-8784-30E7DF222C74}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F49341F-0D7E-4598-9A0A-9D1BA9803DA9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>